<commit_message>
Record Qwen and Kimi judge retry results
</commit_message>
<xml_diff>
--- a/evaluation_multimodels/runs/2026-09-21-minimal32-five-self-included/pairs/claude_claude-opus-5_judge_medium__vs__kimi_kimi-k2.6_judge_high.xlsx
+++ b/evaluation_multimodels/runs/2026-09-21-minimal32-five-self-included/pairs/claude_claude-opus-5_judge_medium__vs__kimi_kimi-k2.6_judge_high.xlsx
@@ -2061,33 +2061,35 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
-        <v>0.001834006980061531</v>
+        <v>10037.70566597814</v>
       </c>
       <c r="M2" t="n">
-        <v>0.008540984708815813</v>
+        <v>2007.110957987607</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2126,33 +2128,35 @@
       <c r="H3" t="b">
         <v>1</v>
       </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>26930.71233300725</v>
+        <v>14639.84687498305</v>
       </c>
       <c r="M3" t="n">
-        <v>0.03362499410286546</v>
+        <v>1073.849874956068</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2191,33 +2195,35 @@
       <c r="H4" t="b">
         <v>1</v>
       </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>12587.97554101329</v>
+        <v>12746.70045799576</v>
       </c>
       <c r="M4" t="n">
-        <v>0.01908402191475034</v>
+        <v>2174.969165993389</v>
       </c>
       <c r="Q4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2256,33 +2262,35 @@
       <c r="H5" t="b">
         <v>1</v>
       </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
-        <v>34817.22745799925</v>
+        <v>15026.58966701711</v>
       </c>
       <c r="M5" t="n">
-        <v>0.009917013812810183</v>
+        <v>1238.939792034216</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2321,33 +2329,35 @@
       <c r="H6" t="b">
         <v>1</v>
       </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
-        <v>0.003083026967942715</v>
+        <v>0.003416964318603277</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0107080559246242</v>
+        <v>3271.607625007164</v>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2386,33 +2396,35 @@
       <c r="H7" t="b">
         <v>1</v>
       </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
-        <v>0.002167013008147478</v>
+        <v>14345.74287501164</v>
       </c>
       <c r="M7" t="n">
-        <v>0.01916603650897741</v>
+        <v>1076.40929101035</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2451,33 +2463,35 @@
       <c r="H8" t="b">
         <v>1</v>
       </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>19507.42441701004</v>
+        <v>13643.43420800287</v>
       </c>
       <c r="M8" t="n">
-        <v>0.005999987479299307</v>
+        <v>1477.751415979583</v>
       </c>
       <c r="Q8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2516,33 +2530,35 @@
       <c r="H9" t="b">
         <v>1</v>
       </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
-        <v>19151.87233302277</v>
+        <v>13510.35170798423</v>
       </c>
       <c r="M9" t="n">
-        <v>0.01520896330475807</v>
+        <v>1772.059999988414</v>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2581,33 +2597,35 @@
       <c r="H10" t="b">
         <v>1</v>
       </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
-        <v>0.002334010787308216</v>
+        <v>0.00604201341047883</v>
       </c>
       <c r="M10" t="n">
-        <v>0.007583003025501966</v>
+        <v>1599.751666013617</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2646,33 +2664,35 @@
       <c r="H11" t="b">
         <v>1</v>
       </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>14601.69974999735</v>
+        <v>14535.09462502552</v>
       </c>
       <c r="M11" t="n">
-        <v>0.01583300763741136</v>
+        <v>1079.051250009798</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2711,33 +2731,35 @@
       <c r="H12" t="b">
         <v>1</v>
       </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
-        <v>112288.2739999914</v>
+        <v>13176.32816697005</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08020800305530429</v>
+        <v>1953.942458028905</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2776,33 +2798,35 @@
       <c r="H13" t="b">
         <v>1</v>
       </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
-        <v>23017.30429101735</v>
+        <v>13834.35474999715</v>
       </c>
       <c r="M13" t="n">
-        <v>0.01662498107179999</v>
+        <v>1150.143667007796</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2841,33 +2865,35 @@
       <c r="H14" t="b">
         <v>1</v>
       </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
-        <v>0.001500011421740055</v>
+        <v>12046.47770797601</v>
       </c>
       <c r="M14" t="n">
-        <v>0.005583977326750755</v>
+        <v>1603.583333024289</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2906,33 +2932,35 @@
       <c r="H15" t="b">
         <v>1</v>
       </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
-        <v>21752.15945800301</v>
+        <v>11676.16491700755</v>
       </c>
       <c r="M15" t="n">
-        <v>0.01054099993780255</v>
+        <v>1346.238875004929</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -2971,33 +2999,35 @@
       <c r="H16" t="b">
         <v>1</v>
       </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
-        <v>0.001707987394183874</v>
+        <v>6428.032000025269</v>
       </c>
       <c r="M16" t="n">
-        <v>0.005709007382392883</v>
+        <v>1667.824916017707</v>
       </c>
       <c r="Q16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -3036,33 +3066,35 @@
       <c r="H17" t="b">
         <v>1</v>
       </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
-        <v>24499.55250002677</v>
+        <v>13811.20716698933</v>
       </c>
       <c r="M17" t="n">
-        <v>0.03095797728747129</v>
+        <v>2135.73754200479</v>
       </c>
       <c r="Q17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>
@@ -3101,33 +3133,35 @@
       <c r="H18" t="b">
         <v>1</v>
       </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
-        <v>10853.94875000929</v>
+        <v>10904.87162501086</v>
       </c>
       <c r="M18" t="n">
-        <v>0.008541042916476727</v>
+        <v>1293.839499994647</v>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["URLError", "URLError"]</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>NOT_ATTEMPTED</t>
+          <t>CONNECTION</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>RuntimeError: TRIAL_CIRCUIT_OPEN_NOT_ATTEMPTED: kimi Judge paused after observed repeated rate limits/timeouts or incomplete streams; prior successful judgements preserved; not a quality zero</t>
+          <t>ProviderCallError: kimi transport failed: URLError: &lt;urlopen error [Errno 8] nodename nor servname provided, or not known&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>